<commit_message>
Direct links to the datasets not repo
</commit_message>
<xml_diff>
--- a/docs/candidate_dataset_register.xlsx
+++ b/docs/candidate_dataset_register.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,11 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="3">
@@ -77,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -85,8 +90,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -458,14 +462,14 @@
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,7 +522,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/jbrownlee/Datasets/blob/master/adult-all.csv</t>
+          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/adult-all.csv</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -539,7 +543,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>workclass 5.7% missing, occupation 5.8% missing, native-country 1.8% missing</t>
+          <t>workclass 5.7% missing, occupation 5.8% missing, native_country 1.8% missing</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -556,7 +560,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>UCI/KEEL, mirror: github.com/jbrownlee/Datasets/blob/master/mammography.csv</t>
+          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/mammography.csv</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -567,7 +571,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Already binary. 1 means calcification found, -1 means not found.</t>
+          <t>Already binary. class 1 means calcification found, -1 means not found.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -594,7 +598,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>kaggle.com/datasets/mlg-ulb/creditcardfraud</t>
+          <t>https://www.kaggle.com/datasets/mlg-ulb/creditcardfraud</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -632,7 +636,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>archive.ics.uci.edu/dataset/222/bank+marketing</t>
+          <t>https://raw.githubusercontent.com/khatrideepti/Bank-Marketing-Data-Analysis/master/bank-full.csv</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -670,7 +674,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>kaggle.com/c/GiveMeSomeCredit</t>
+          <t>https://raw.githubusercontent.com/JLZml/Credit-Scoring-Data-Sets/master/3.%20Kaggle/Give%20Me%20Some%20Credit/cs-training.csv</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -700,7 +704,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>MAGIC Gamma Telescope</t>
@@ -708,7 +712,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/mikeizbicki/datasets/blob/master/csv/uci/magic04.data</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/magic04.data</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -719,7 +723,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Already binary. g means gamma ray, h means hadron.</t>
+          <t>Already binary. class g means gamma ray, h means hadron.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -734,11 +738,11 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Online Shoppers Purchasing Intention</t>
@@ -746,7 +750,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/sharmaroshan/Online-Shoppers-Purchasing-Intention</t>
+          <t>https://raw.githubusercontent.com/sharmaroshan/Online-Shoppers-Purchasing-Intention/master/online_shoppers_intention.csv</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -776,7 +780,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>EEG Eye State</t>
@@ -784,7 +788,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/Krishh-mishra98/eeg-eye-state-dataset</t>
+          <t>https://raw.githubusercontent.com/Krishh-mishra98/eeg-eye-state-dataset/master/eeg.csv</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -795,7 +799,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Already binary. 1 means eyes closed, 2 means eyes open (we treat this as 0/1).</t>
+          <t>Already binary. 1 means eyes closed, 2 means eyes open (treated as 0/1).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -814,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="55" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Rain in Australia (weatherAUS)</t>
@@ -822,7 +826,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kaggle: kaggle.com/datasets/jsphyg/weather-dataset-rattle-package, mirror: github.com/acakin/weatherAUS</t>
+          <t>https://raw.githubusercontent.com/acakin/weatherAUS/master/weatherAUS.csv</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -852,11 +856,11 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>From the Australian Bureau of Meteorology, shared on Kaggle. Check the Kaggle page for the exact reuse terms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+          <t>From the Australian Bureau of Meteorology, shared on Kaggle. Check the Kaggle page for exact reuse terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Diabetes 130-US Hospitals</t>
@@ -864,7 +868,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/swengzju/Predicting-Diabetes-Patient-Readmission</t>
+          <t>https://raw.githubusercontent.com/swengzju/Predicting-Diabetes-Patient-Readmission/master/diabetic_data.csv</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -877,7 +881,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Was 3 classes (NO, &lt;30, &gt;30 days). We made it binary: 1 = readmitted in under 30 days, 0 = not.</t>
+          <t>Was 3 classes (NO, &lt;30, &gt;30 days). Made binary: 1 = readmitted in under 30 days, 0 = not.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -904,7 +908,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/mikeizbicki/datasets/blob/master/csv/uci/letter-recognition.data</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/letter-recognition.data</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -915,7 +919,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Was 26 classes (one per letter). We made it binary: 1 = vowel (A, E, I, O, U), 0 = consonant.</t>
+          <t>Was 26 classes (one per letter). Made binary: 1 = vowel (A, E, I, O, U), 0 = consonant.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -930,7 +934,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
         </is>
       </c>
     </row>
@@ -942,7 +946,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/ducanng/Decision-Tree-with-scikit-learn/blob/master/connect-4.data</t>
+          <t>https://raw.githubusercontent.com/ducanng/Decision-Tree-with-scikit-learn/master/connect-4.data</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -953,7 +957,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Was 3 classes (win, loss, draw). We made it binary: 1 = win, 0 = not a win (loss or draw).</t>
+          <t>Was 3 classes (win, loss, draw). Made binary: 1 = win, 0 = not a win.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -968,7 +972,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
         </is>
       </c>
     </row>
@@ -980,7 +984,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/mikeizbicki/datasets/blob/master/csv/uci/shuttle.tst</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/shuttle.tst</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -991,7 +995,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Was 7 classes. We made it binary: 1 = class 1 'Rad Flow', 0 = any other class.</t>
+          <t>Was 7 classes. Made binary: 1 = class 1 "Rad Flow", 0 = any other class.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1006,7 +1010,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: this is only the test portion of the full Statlog Shuttle dataset (the full set has about 58,000 rows). We could only get this file, so numbers here are for this 14,500-row file only.</t>
+          <t>CC BY 4.0. Note: this is only the test portion of the full dataset (the full set has about 58,000 rows). File ends in .tst, not .csv, but it's plain space-separated text that opens fine in Excel or pandas.</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1022,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/mikeizbicki/datasets/blob/master/csv/uci/nursery.data</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/nursery.data</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1029,7 +1033,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Was 5 classes. We made it binary: 1 = not_recom (application not recommended), 0 = any other outcome.</t>
+          <t>Was 5 classes. Made binary: 1 = not_recom (application not recommended), 0 = any other outcome.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1044,7 +1048,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1060,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>UCI, mirror: github.com/mikeizbicki/datasets/blob/master/csv/uci/krkopt.data</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/krkopt.data</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1067,7 +1071,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Was 18 classes (draw, or number of moves to win). We made it binary: 1 = draw, 0 = White wins in some number of moves.</t>
+          <t>Was 18 classes (draw, or number of moves to win). Made binary: 1 = draw, 0 = White wins in some number of moves.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1082,7 +1086,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
         </is>
       </c>
     </row>
@@ -1272,34 +1276,44 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>I looked at 24 datasets in total across all rounds. 15 made it in, 9 did not.</t>
         </is>
       </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Main reason for rejecting: too few rows (6 out of 9).</t>
         </is>
       </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Other reason: could not find a working download link to check the numbers ourselves (3 out of 9: Default of Credit Card Clients, Covertype, HTRU2).</t>
         </is>
       </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1310,7 +1324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1422,6 +1436,21 @@
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>For Statlog Shuttle, we could only get the 14,500-row test file, not the full ~58,000-row dataset. We used it anyway since it clears the 10,000-row minimum on its own, but we wrote clearly that it's only part of the full dataset so nobody assumes we checked the whole thing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Some of our first links pointed to a whole GitHub repo instead of the actual file, and one link (weatherAUS) looked broken when we first checked it.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>We re-checked every link and replaced each one with the exact raw file URL (the direct link to the file itself, not the repo page). All 15 now point straight at a working file. We tried uploading the actual data into this repo too, but GitHub rejected some files for being too large, so we kept this as links only, same as the assignment allows.</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1444,33 +1473,27 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Hardest rule to follow and why</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="n"/>
+    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>The hardest rule was checking the row count myself. It sounds simple, but two datasets I wanted to use (Default of Credit Card Clients and Covertype) could not be downloaded in this session, so I could not open the file and count the rows myself. I did not want to just use the number from the dataset page, since that is exactly what the assignment says not to do, so I left both out instead. The other tricky part was missing data. Bank Marketing has a column that is mostly filled with the word 'unknown,' and it was not obvious if that should count as missing data or not.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>The hardest rule was checking the row count ourselves. It's simple once you have the file, but some datasets we wanted (Default of Credit Card Clients, Covertype, HTRU2) couldn't be downloaded in the time we had, so we couldn't open the file and count the rows ourselves. Rather than just use the number from the dataset page, which is exactly what the assignment says not to do, we left those out. We also had a link problem partway through: a couple of our early links pointed at a whole GitHub repo instead of the actual file, and one looked dead. We fixed that by re-checking every single link and replacing it with the exact raw file URL, so every source in this register points straight at a working file, not a repo homepage. The other tricky part was missing data and picking a binarisation rule -- several datasets that fit everything else had a few columns that were mostly missing (Rain in Australia, Diabetes 130-US Hospitals), so we had to decide to drop those specific columns rather than the whole dataset, and several others (Letter Recognition, Connect-4, Nursery, Chess, Shuttle) had more than two classes, so we had to pick and write down exactly which class counted as the positive one.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A3:E10"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Links correction direct download
</commit_message>
<xml_diff>
--- a/docs/candidate_dataset_register.xlsx
+++ b/docs/candidate_dataset_register.xlsx
@@ -463,13 +463,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,7 +522,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/adult-all.csv</t>
+          <t>https://archive.ics.uci.edu/static/public/2/adult.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/mammography.csv</t>
+          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/mammography.csv (opens as text in browser -- use Ctrl+S / Save Page As to save it, or right-click the link and choose Save Link As)</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -598,7 +598,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaggle.com/datasets/mlg-ulb/creditcardfraud</t>
+          <t>https://www.kaggle.com/datasets/mlg-ulb/creditcardfraud (click the Download button on the page -- needs a free Kaggle account)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -636,7 +636,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/khatrideepti/Bank-Marketing-Data-Analysis/master/bank-full.csv</t>
+          <t>https://archive.ics.uci.edu/static/public/222/bank+marketing.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -674,7 +674,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/JLZml/Credit-Scoring-Data-Sets/master/3.%20Kaggle/Give%20Me%20Some%20Credit/cs-training.csv</t>
+          <t>https://www.kaggle.com/c/GiveMeSomeCredit/data (click the Download button on the page -- needs a free Kaggle account)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -712,7 +712,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/magic04.data</t>
+          <t>https://archive.ics.uci.edu/static/public/159/magic+gamma+telescope.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -738,7 +738,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/sharmaroshan/Online-Shoppers-Purchasing-Intention/master/online_shoppers_intention.csv</t>
+          <t>https://archive.ics.uci.edu/static/public/468/online+shoppers+purchasing+intention+dataset.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Krishh-mishra98/eeg-eye-state-dataset/master/eeg.csv</t>
+          <t>https://archive.ics.uci.edu/static/public/264/eeg+eye+state.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -826,7 +826,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/acakin/weatherAUS/master/weatherAUS.csv</t>
+          <t>https://www.kaggle.com/datasets/jsphyg/weather-dataset-rattle-package (click the Download button on the page -- needs a free Kaggle account)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/swengzju/Predicting-Diabetes-Patient-Readmission/master/diabetic_data.csv</t>
+          <t>https://archive.ics.uci.edu/static/public/296/diabetes+130-us+hospitals+for+years+1999-2008.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/letter-recognition.data</t>
+          <t>https://archive.ics.uci.edu/static/public/59/letter+recognition.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -934,7 +934,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/ducanng/Decision-Tree-with-scikit-learn/master/connect-4.data</t>
+          <t>https://archive.ics.uci.edu/static/public/26/connect+4.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -972,7 +972,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/shuttle.tst</t>
+          <t>https://archive.ics.uci.edu/static/public/148/statlog+shuttle.zip (click to download directly -- zip has both train and test files, we only checked the test file)</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: this is only the test portion of the full dataset (the full set has about 58,000 rows). File ends in .tst, not .csv, but it's plain space-separated text that opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0. Note: we only checked the numbers for the 14,500-row test file inside the zip, not the full ~58,000-row training file.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/nursery.data</t>
+          <t>https://archive.ics.uci.edu/static/public/76/nursery.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/krkopt.data</t>
+          <t>https://archive.ics.uci.edu/static/public/22/chess+king+rook+vs+king.zip (click to download directly)</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: file ends in .data, not .csv, but it's plain comma-separated text and opens fine in Excel or pandas.</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1445,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Some of our first links pointed to a whole GitHub repo instead of the actual file, and one link (weatherAUS) looked broken when we first checked it.</t>
+          <t>Our GitHub raw links pointed at the right file, but clicking them just opens a wall of text in the browser instead of downloading anything -- that's how GitHub serves raw files, not a broken link.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>We re-checked every link and replaced each one with the exact raw file URL (the direct link to the file itself, not the repo page). All 15 now point straight at a working file. We tried uploading the actual data into this repo too, but GitHub rejected some files for being too large, so we kept this as links only, same as the assignment allows.</t>
+          <t>For every dataset that lives on UCI, we switched to UCI's own official Download button link (a .zip file that actually downloads when clicked). For the two that only exist on Kaggle, we pointed to the page's Download button (needs a free Kaggle login, but that's a real download, not a text dump). Mammography doesn't have an official zip anywhere, so we kept the GitHub link but wrote in the register that you need to use Ctrl+S or Save Link As to save it, since simply clicking it just displays the text.</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>The hardest rule was checking the row count ourselves. It's simple once you have the file, but some datasets we wanted (Default of Credit Card Clients, Covertype, HTRU2) couldn't be downloaded in the time we had, so we couldn't open the file and count the rows ourselves. Rather than just use the number from the dataset page, which is exactly what the assignment says not to do, we left those out. We also had a link problem partway through: a couple of our early links pointed at a whole GitHub repo instead of the actual file, and one looked dead. We fixed that by re-checking every single link and replacing it with the exact raw file URL, so every source in this register points straight at a working file, not a repo homepage. The other tricky part was missing data and picking a binarisation rule -- several datasets that fit everything else had a few columns that were mostly missing (Rain in Australia, Diabetes 130-US Hospitals), so we had to decide to drop those specific columns rather than the whole dataset, and several others (Letter Recognition, Connect-4, Nursery, Chess, Shuttle) had more than two classes, so we had to pick and write down exactly which class counted as the positive one.</t>
+          <t>The hardest rule was checking the row count ourselves. It's simple once you have the file, but some datasets we wanted (Default of Credit Card Clients, Covertype, HTRU2) couldn't be downloaded in the time we had, so we couldn't open the file and count the rows ourselves. Rather than just use the number from the dataset page, which is exactly what the assignment says not to do, we left those out. We also had a link problem partway through: several of our links technically worked but just opened as a wall of text in the browser instead of downloading anything, since that's how GitHub serves raw files. We fixed this by switching every UCI-hosted dataset to UCI's own official Download button link, which actually saves a file, and by pointing the two Kaggle datasets at their page's Download button instead. The other tricky part was missing data and picking a binarisation rule -- several datasets that fit everything else had a few columns that were mostly missing (Rain in Australia, Diabetes 130-US Hospitals), so we had to decide to drop those specific columns rather than the whole dataset, and several others (Letter Recognition, Connect-4, Nursery, Chess, Shuttle) had more than two classes, so we had to pick and write down exactly which class counted as the positive one.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MOre fixes on datasets link
</commit_message>
<xml_diff>
--- a/docs/candidate_dataset_register.xlsx
+++ b/docs/candidate_dataset_register.xlsx
@@ -469,7 +469,7 @@
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,7 +514,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="55" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Adult Income</t>
@@ -522,7 +522,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/2/adult.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/adult-all.csv</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -552,7 +552,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="55" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Mammography</t>
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/mammography.csv (opens as text in browser -- use Ctrl+S / Save Page As to save it, or right-click the link and choose Save Link As)</t>
+          <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/mammography.csv (opens as text in browser -- use Ctrl+S / Save Page As to save it)</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -590,7 +590,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="55" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Credit Card Fraud</t>
@@ -598,7 +598,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaggle.com/datasets/mlg-ulb/creditcardfraud (click the Download button on the page -- needs a free Kaggle account)</t>
+          <t>https://www.kaggle.com/datasets/mlg-ulb/creditcardfraud (click the Download button on the page -- needs a free Kaggle account, downloads as a single csv since it's a single-file dataset)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -628,7 +628,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="55" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Bank Marketing</t>
@@ -636,7 +636,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/222/bank+marketing.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/khatrideepti/Bank-Marketing-Data-Analysis/master/bank-full.csv</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -666,7 +666,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Give Me Some Credit</t>
@@ -674,7 +674,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaggle.com/c/GiveMeSomeCredit/data (click the Download button on the page -- needs a free Kaggle account)</t>
+          <t>https://www.kaggle.com/c/GiveMeSomeCredit/data (click the Download button on the page -- needs a free Kaggle account, downloads as a single csv since it's a single-file dataset)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -704,7 +704,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="55" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>MAGIC Gamma Telescope</t>
@@ -712,7 +712,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/159/magic+gamma+telescope.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/EpistasisLab/tpot/master/tutorials/MAGIC%20Gamma%20Telescope/MAGIC%20Gamma%20Telescope%20Data.csv</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Online Shoppers Purchasing Intention</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/468/online+shoppers+purchasing+intention+dataset.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/sharmaroshan/Online-Shoppers-Purchasing-Intention/master/online_shoppers_intention.csv</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -780,7 +780,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="55" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>EEG Eye State</t>
@@ -788,7 +788,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/264/eeg+eye+state.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/Krishh-mishra98/eeg-eye-state-dataset/master/eeg.csv</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -818,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="55" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Rain in Australia (weatherAUS)</t>
@@ -826,7 +826,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaggle.com/datasets/jsphyg/weather-dataset-rattle-package (click the Download button on the page -- needs a free Kaggle account)</t>
+          <t>https://raw.githubusercontent.com/acakin/weatherAUS/master/weatherAUS.csv</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="55" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Diabetes 130-US Hospitals</t>
@@ -868,7 +868,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/296/diabetes+130-us+hospitals+for+years+1999-2008.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/swengzju/Predicting-Diabetes-Patient-Readmission/master/diabetic_data.csv</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -900,7 +900,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="55" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Letter Recognition</t>
@@ -908,7 +908,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/59/letter+recognition.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/aiez/klassif/main/letter.csv</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -934,11 +934,11 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="55" customHeight="1">
+          <t>CC BY 4.0 (original UCI data). This particular csv copy is shared under MIT by the repo maintainer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Connect-4</t>
@@ -946,7 +946,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/26/connect+4.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/ducanng/Decision-Tree-with-scikit-learn/master/connect-4.data (opens as text in browser -- use Ctrl+S / Save Page As to save it)</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -972,11 +972,11 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="55" customHeight="1">
+          <t>CC BY 4.0. Note: we searched for a plain .csv version of this one and couldn't find a working one, so this is a .data file -- same single comma-separated file, just an older file extension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Statlog Shuttle (test split)</t>
@@ -984,7 +984,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/148/statlog+shuttle.zip (click to download directly -- zip has both train and test files, we only checked the test file)</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/shuttle.tst (opens as text in browser -- use Ctrl+S / Save Page As to save it)</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1010,11 +1010,11 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0. Note: we only checked the numbers for the 14,500-row test file inside the zip, not the full ~58,000-row training file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="55" customHeight="1">
+          <t>CC BY 4.0. Note: this is only the test portion of the full dataset (the full set has about 58,000 rows). We searched for a plain .csv version and couldn't find one, so this is a .tst file -- same single space-separated file, just an older file extension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Nursery</t>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/76/nursery.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/aiez/klassif/main/nursery.csv</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1048,11 +1048,11 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="55" customHeight="1">
+          <t>CC BY 4.0 (original UCI data). This particular csv copy is shared under MIT by the repo maintainer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chess (King-Rook vs King)</t>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://archive.ics.uci.edu/static/public/22/chess+king+rook+vs+king.zip (click to download directly)</t>
+          <t>https://raw.githubusercontent.com/mikeizbicki/datasets/master/csv/uci/krkopt.data (opens as text in browser -- use Ctrl+S / Save Page As to save it)</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>CC BY 4.0. Note: we searched for a plain .csv version of this one and couldn't find one -- there's a similarly-named 'King-Rook vs King-Pawn' dataset out there but it's a different dataset with far fewer rows, so we didn't substitute it. This is a .data file -- same single comma-separated file, just an older file extension.</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>The hardest rule was checking the row count ourselves. It's simple once you have the file, but some datasets we wanted (Default of Credit Card Clients, Covertype, HTRU2) couldn't be downloaded in the time we had, so we couldn't open the file and count the rows ourselves. Rather than just use the number from the dataset page, which is exactly what the assignment says not to do, we left those out. We also had a link problem partway through: several of our links technically worked but just opened as a wall of text in the browser instead of downloading anything, since that's how GitHub serves raw files. We fixed this by switching every UCI-hosted dataset to UCI's own official Download button link, which actually saves a file, and by pointing the two Kaggle datasets at their page's Download button instead. The other tricky part was missing data and picking a binarisation rule -- several datasets that fit everything else had a few columns that were mostly missing (Rain in Australia, Diabetes 130-US Hospitals), so we had to decide to drop those specific columns rather than the whole dataset, and several others (Letter Recognition, Connect-4, Nursery, Chess, Shuttle) had more than two classes, so we had to pick and write down exactly which class counted as the positive one.</t>
+          <t>The hardest rule was checking the row count ourselves. It's simple once you have the file, but some datasets we wanted (Default of Credit Card Clients, Covertype, HTRU2) couldn't be downloaded in the time we had, so we couldn't open the file and count the rows ourselves. Rather than just use the number from the dataset page, which is exactly what the assignment says not to do, we left those out. We also went through two rounds of link problems: first, some links pointed at a repo instead of a file, or opened as a wall of text instead of downloading; then, once we fixed that, we still wanted single .csv files with no zip to extract, so we went back and found real .csv mirrors for three more datasets (MAGIC, Letter Recognition, Nursery). Three others (Connect-4, Statlog Shuttle, Chess King-Rook vs King) still don't have a .csv version we could find, so those stay as .data/.tst files -- still a single file, just an older extension. The other tricky part was missing data and picking a binarisation rule -- several datasets that fit everything else had a few columns that were mostly missing (Rain in Australia, Diabetes 130-US Hospitals), so we had to decide to drop those specific columns rather than the whole dataset, and several others (Letter Recognition, Connect-4, Nursery, Chess, Shuttle) had more than two classes, so we had to pick and write down exactly which class counted as the positive one.</t>
         </is>
       </c>
     </row>

</xml_diff>